<commit_message>
Updated JOR model - 2025-11-25 09:48
</commit_message>
<xml_diff>
--- a/VerveStacks_JOR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JOR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JOR\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7435461-178E-4451-B003-C278E7879A67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{805BF89B-23C5-4580-914B-01F4D0FC83A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5639,7 +5639,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{559EA8A7-CBB9-43C3-A675-D2E9B4E2B4E9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68E01723-67BC-463F-A89E-EC348A80DDCA}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6042,7 +6042,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F11A44D1-B784-4760-8210-681752C2492E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9DA4F44-92C0-4C4D-9E94-D4D18F171B78}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6445,7 +6445,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69015E6D-36E1-49FB-BA19-128ED15EE081}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2476C8-9A75-4222-8B0B-01C6C98C5C10}">
   <dimension ref="B9:P64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>